<commit_message>
Traceability shows 'assumed' coverage (tested, but the criterion has an open gap); wireframes for gap triage, traceability and evaluation dashboard
</commit_message>
<xml_diff>
--- a/outputs/PRD-1.1_cleaning_log_and_rejection/test_library_v1.0.xlsx
+++ b/outputs/PRD-1.1_cleaning_log_and_rejection/test_library_v1.0.xlsx
@@ -32,7 +32,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -49,6 +49,11 @@
         <fgColor rgb="00FCE4E4"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF4E0"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -62,13 +67,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -485,7 +493,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>23 test cases drafted, 14 requirement gaps raised, 1 criteria without a test case</t>
+          <t>23 test cases drafted, 14 requirement gaps raised, 1 criteria without a test case, 2 tested on an assumption</t>
         </is>
       </c>
     </row>
@@ -2253,62 +2261,62 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>US-104</t>
         </is>
       </c>
-      <c r="B10" s="2" t="n">
+      <c r="B10" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>QA can override as needed.</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>TC-104-01, TC-104-02, TC-104-03, TC-104-04</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>vague_term, gxp_control_missing</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>assumed</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>US-105</t>
         </is>
       </c>
-      <c r="B11" s="2" t="n">
+      <c r="B11" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>The report shows cleanings. TBD which filters.</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>TC-105-01, TC-105-02, TC-105-03, TC-105-04</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>placeholder</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>assumed</t>
         </is>
       </c>
     </row>

</xml_diff>